<commit_message>
changed add task from file to json string
</commit_message>
<xml_diff>
--- a/расчет батча.xlsx
+++ b/расчет батча.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Grid Calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99B990A3-3C5D-454C-A095-76A0A8553F92}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B257F9EF-4CDC-42D1-8B8E-0DCCC0E0D425}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F4793AFB-05E6-43C9-9995-743683279B2A}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>белые</t>
   </si>
@@ -58,12 +58,24 @@
   </si>
   <si>
     <t>огр. по инту</t>
+  </si>
+  <si>
+    <t>огр. по лонгу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">макс - </t>
+  </si>
+  <si>
+    <t>&gt; 30 мин</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -103,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -112,6 +124,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -430,126 +446,167 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
-    <col min="7" max="7" width="40.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="32.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <f>12^B2</f>
+      <c r="B2" s="1">
+        <f>12^C2</f>
         <v>1.5407021574586368E+16</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>15</v>
       </c>
-      <c r="C2" s="1">
-        <f>4^D2</f>
+      <c r="D2" s="1">
+        <f>4^E2</f>
         <v>65536</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>8</v>
       </c>
-      <c r="E2" s="1">
-        <f>A2*C2</f>
+      <c r="F2" s="1">
+        <f>B2*D2</f>
         <v>1.0097145659120922E+21</v>
       </c>
-      <c r="F2" s="1">
-        <f>E2/E3</f>
-        <v>322486272</v>
-      </c>
       <c r="G2" s="1">
-        <f>F2*G3/60/60</f>
-        <v>1791.5904000000003</v>
-      </c>
-      <c r="H2">
-        <f>G2/100</f>
-        <v>17.915904000000001</v>
+        <f>F2/F3</f>
+        <v>8916100448256</v>
+      </c>
+      <c r="H2" s="5">
+        <f>G2*H3/60/60</f>
+        <v>619173642240</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <f>12^B3</f>
-        <v>2985984</v>
-      </c>
-      <c r="B3">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <f>4^D3</f>
-        <v>1048576</v>
-      </c>
-      <c r="D3">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1">
-        <f>A3*C3</f>
-        <v>3131031158784</v>
-      </c>
-      <c r="F3" s="1" t="b">
-        <f>F2&lt;=A8</f>
+      <c r="B3" s="1">
+        <f>12^C3</f>
+        <v>1728</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1">
+        <f>4^E3</f>
+        <v>65536</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3" s="1">
+        <f>B3*D3</f>
+        <v>113246208</v>
+      </c>
+      <c r="H3" s="5">
+        <f>250</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="b">
+        <f>B3&lt;=A5</f>
         <v>1</v>
       </c>
-      <c r="G3" s="1">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="b">
-        <f>A3&lt;=A8</f>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1" t="b">
+        <f>D3&lt;=A5</f>
         <v>1</v>
       </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="1" t="b">
-        <f>C3&lt;=A8</f>
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="b">
+        <f>G2&lt;=A5</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F5" s="1"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
+      <c r="A5" s="1">
         <f>2^31-1</f>
         <v>2147483647</v>
       </c>
+      <c r="B5" s="1"/>
+      <c r="C5"/>
+      <c r="D5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="b">
+        <f>B3&lt;=A7</f>
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="b">
+        <f>D3&lt;=A7</f>
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" t="b">
+        <f>G2&lt;=A7</f>
+        <v>1</v>
+      </c>
+      <c r="H6" s="5"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <f>2^63-1</f>
+        <v>9.2233720368547758E+18</v>
+      </c>
+      <c r="C7"/>
+      <c r="D7" s="1"/>
+      <c r="G7"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C8"/>
+      <c r="D8" s="1"/>
+      <c r="G8"/>
+      <c r="H8" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
beginning of implementation of looping batches
</commit_message>
<xml_diff>
--- a/расчет батча.xlsx
+++ b/расчет батча.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Grid Calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{056F25F8-F3AD-48B0-8F83-F69D3EF262F3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8AD9860-6A17-4774-96A5-AF41B8B14FFC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F4793AFB-05E6-43C9-9995-743683279B2A}"/>
   </bookViews>
@@ -600,6 +600,10 @@
         <f>2^63-1</f>
         <v>9.2233720368547758E+18</v>
       </c>
+      <c r="B7" t="b">
+        <f>B2&lt;=A7</f>
+        <v>1</v>
+      </c>
       <c r="C7"/>
       <c r="D7" s="1"/>
       <c r="G7"/>

</xml_diff>